<commit_message>
fix pipeline, class README.md & merge notebook
</commit_message>
<xml_diff>
--- a/src/result/lfw/model_comparison.xlsx
+++ b/src/result/lfw/model_comparison.xlsx
@@ -483,16 +483,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.659515142440796</v>
+        <v>1.406541347503662</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06751608848571777</v>
+        <v>0.05563020706176758</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1856036186218262</v>
+        <v>0.1125195026397705</v>
       </c>
       <c r="E4" t="n">
-        <v>6.051357269287109</v>
+        <v>7.665030241012573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix module and pipeline, add comments & fix README.md
</commit_message>
<xml_diff>
--- a/src/result/lfw/model_comparison.xlsx
+++ b/src/result/lfw/model_comparison.xlsx
@@ -483,16 +483,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.406541347503662</v>
+        <v>1.536517143249512</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05563020706176758</v>
+        <v>0.05829548835754395</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1125195026397705</v>
+        <v>0.09912467002868652</v>
       </c>
       <c r="E4" t="n">
-        <v>7.665030241012573</v>
+        <v>8.332909345626831</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: aggiunti benchmark pre-SVD, test Unknown ed esplicitate metriche
- Implementato test dei classificatori sui dati raw senza SVD.
- Aggiunta validazione dell'Unknown Detection sul test set (FRR misurato al 3% tramite distanza Euclidea).
- Esplicitate le metriche in compare_classifiers (Accuracy, Precision, Recall, F1).
</commit_message>
<xml_diff>
--- a/src/result/lfw/model_comparison.xlsx
+++ b/src/result/lfw/model_comparison.xlsx
@@ -413,86 +413,100 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E1" t="n">
-        <v>3</v>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>f1_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
           <t>KNN</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>SVM Linear</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>SVM RBF</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>SVM Best</t>
-        </is>
+      <c r="B2" t="n">
+        <v>0.6201780415430267</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.6300128136811414</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.6201780415430267</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.6197418518232976</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.02699756622314453</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>SVM Linear</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.6201780415430267</v>
+        <v>0.8100890207715133</v>
       </c>
       <c r="C3" t="n">
+        <v>0.8222371908425218</v>
+      </c>
+      <c r="D3" t="n">
         <v>0.8100890207715133</v>
       </c>
-      <c r="D3" t="n">
-        <v>0.798219584569733</v>
-      </c>
       <c r="E3" t="n">
-        <v>0.8041543026706232</v>
+        <v>0.8114621599894675</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.2565765380859375</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>SVM RBF</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.536517143249512</v>
+        <v>0.798219584569733</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05829548835754395</v>
+        <v>0.7994274271722341</v>
       </c>
       <c r="D4" t="n">
-        <v>0.09912467002868652</v>
+        <v>0.798219584569733</v>
       </c>
       <c r="E4" t="n">
-        <v>8.332909345626831</v>
+        <v>0.7937009641150342</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.4562253952026367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>